<commit_message>
feat(warroom): reset all 10 leads to start point and enable full in-drawer editing
</commit_message>
<xml_diff>
--- a/public/pfg_b2b_tracker.xlsx
+++ b/public/pfg_b2b_tracker.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>در حال بررسی</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -665,17 +665,17 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>پیش‌نویس آماده</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>در انتظار بررسی</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>آماده‌سازی پکیج تست ۵۰ هزارتایی و هماهنگی جلسه فنی</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>تکمیل شده</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -732,17 +732,17 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>پیش‌نویس آماده</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>ورود مستقیم مدیرعامل</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>هماهنگی جلسه در سطح مدیران عامل با هلدینگ حصین</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>تکمیل شده</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -799,17 +799,17 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>در حال نگارش</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>در انتظار بررسی</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>ارائه آفر پایلوت بدون ریسک و تمرکز بر پشتیبانی شبانه</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>در حال بررسی</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -866,17 +866,17 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>در انتظار اطلاعات</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>ورود مدیرعامل / COO</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>بررسی ارتباطات هلدینگی سنا گستر سبز و حرکت اول</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>تکمیل شده</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -933,17 +933,17 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>پیش‌نویس آماده</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>تایید شد</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>طرح مدل تسهیم سود (Revenue Share 50-50) در نسخه استاندارد</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>تکمیل شده</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
@@ -1000,17 +1000,17 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>پیش‌نویس رسمی</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>ورود مستقیم مدیرعامل</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>مذاکره صنفی / حاکمیتی جهت افزودن وب‌سرویس در هسته نرم‌افزار</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>در حال بررسی</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1067,17 +1067,17 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>در حال نگارش</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>در انتظار بررسی</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>ارسال پیام دمو وب‌هوک به تیم فنی دانشگاه شریف</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>در حال بررسی</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
@@ -1134,17 +1134,17 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>پیش‌نویس آماده</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>در انتظار بررسی</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>پیگیری مذاکره بر مبنای کاهش نرخ نکول و پیامک‌های سررسید</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>تکمیل شده</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1201,17 +1201,17 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>در حال نگارش</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>در انتظار بررسی</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>تاکید بر وب‌هوک معتبر قضایی و گزارش تحویل تا گوشی</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>تکمیل شده</t>
+          <t>شروع نشده (آماده ویرایش)</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
@@ -1268,17 +1268,17 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>پیش‌نویس آماده</t>
+          <t>در انتظار تدوین نامه</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>در انتظار بررسی</t>
+          <t>در انتظار پیش‌نویس</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>پیشنهاد تخفیف پله‌ای بر اساس حجم میلیونی بارکدها</t>
+          <t>کشف و ارزیابی لید (Prospect)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(warroom): assign 4 explicit operational roles (Mrs. Shahroozi, Mrs. Moosapour, Mrs. Khordamdel, Mrs. Faeze)
</commit_message>
<xml_diff>
--- a/public/pfg_b2b_tracker.xlsx
+++ b/public/pfg_b2b_tracker.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>مسئول تحقیق لینکدین (عضو ۱)</t>
+          <t>سرپرست عملیات (خانم خرسنددل)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>مسئول نگارش نامه و مسیرها (عضو ۲)</t>
+          <t>ادمین عملیات (خانم فائزه)</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>تایید مدیریت ارشد (CEO / COO)</t>
+          <t>تایید مدیر ارشد عملیات و مدیرعامل (خانم موسی‌پور / خانم شهروزی)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>همکار ۱ (تیم لینکدین)</t>
+          <t>خانم خرسنددل (Operation Lead)</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>همکار ۲ (تیم محتوا/نامه)</t>
+          <t>خانم فائزه (Operation Admin)</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>در انتظار پیش‌نویس</t>
+          <t>در انتظار بررسی COO/CEO</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
@@ -2397,7 +2397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2436,80 +2436,102 @@
       </c>
     </row>
     <row r="3" ht="55" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>همکار ۱: مسئول تحقیق لینکدین (LinkedIn Researcher)</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>• جستجوی پروفایل‌های کارکنان و مدیران ۱۰ شرکت کاندیدا در لینکدین
-• استخراج نام دقیق و لینک پروفایل مدیران عامل، CTOها و مدیران محصول
-• شناسایی کانکشن‌های مشترک (Mutual Connections) با سرکار خانم شهروزی و سرکار خانم موسی‌پور
-• به‌روزرسانی ستون 'وضعیت تحقیق لینکدین' در شیت اول</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn Sales Navigator / Jobinja / Quera
-خروجی: پر کردن ستون پروفایل‌های افراد در شیت ۲</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>تکمیل اطلاعات ۲ شرکت در روز (پوشش کامل ۱۰ شرکت ظرف ۵ روز)</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>سرکار خانم سوده شهروزی (مدیرعامل / CEO)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>• هدایت کلان استراتژی نفوذ در هلدینگ‌ها و رهبری توافقات کلیدی سازمانی
+• گشایش ارتباط با هیئت‌مدیره کاندیداها از طریق ظرفیت سازمان نصر
+• تصویب نهایی تفاهم‌نامه‌های سازمانی و مدل تسهیم درآمد (Revenue Share)
+• چراغ سبز نهایی آغاز پایلوت فنی رایگان</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>بورد اختصاصی War Room، جلسات شورای راهبری، مکاتبات C-Level</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>تایید و تعیین مسیر ۲ اکانت استراتژیک در هفته</t>
         </is>
       </c>
     </row>
     <row r="4" ht="55" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>همکار ۲: مسئول نگارش نامه و روت‌ها (Contact Letter &amp; Route Drafter)</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>• شخصی‌سازی قلاب‌های متنی شیت ۳ برای هر شخص بر اساس دستاوردهای اخیر آن شرکت
-• تنظیم متن کامل نامه رسمی یا پیام مستقیم (InMail/Email)
-• آماده‌سازی پروپوزال متناسب با نوع ورود (تست ۵۰ هزارتایی یا مدل ری‌شیرینگ)
-• ثبت پیش‌نویس نهایی و تغییر وضعیت به 'پیش‌نویس آماده' در شیت ۱</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Microsoft Word / قالب‌های رسمی پرشیا فاوا / ابزار هوش مصنوعی Gemini
-خروجی: پیش‌نویس متن نهایی نامه و پیام</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>نگارش و آماده‌سازی روزانه ۲ پیش‌نویس نهایی جهت بررسی</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>سرکار خانم مریم موسی‌پور (مدیر ارشد عملیات / COO)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>• راهبری عملیاتی فرآیند فروش و نظارت بر انطباق روت‌های پیامک با SLA تضمینی
+• تایید پیش‌نویس بسته‌های پیشنهادی و تعیین ساختار تعرفه اقتصادی پلکانی
+• پایش پیشرفت روزانه کارت‌ها در تخته کانبان و رفع موانع اتصال فنی
+• نظارت بر حسن انجام تعهدات تیم عملیات</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>بورد آنلاین، کاربرگ جامع اکسل، گزارش‌های ترافیک SMPP</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>بررسی روزانه ساعت ۱۶:۰۰ و تایید نامه‌ها و پیش‌نویس‌ها</t>
         </is>
       </c>
     </row>
     <row r="5" ht="55" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>مدیریت ارشد (CEO / COO Review Gate)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>• بررسی و تایید پیش‌نویس پیام‌ها و نامه‌های آماده‌شده
-• تصمیم‌گیری درباره نحوه ارسال (آیا مستقیماً با امضای مدیرعامل ارسال شود یا توسط تیم تجاری)
-• هماهنگی تماس‌های تلفنی سطح ۱ با اعضای هیئت‌مدیره هلدینگ‌های هدف (نظیر حصین و سنا گستر)
-• تغییر ستون 'تایید مدیریت ارشد' به 'تایید شد' یا 'ورود مستقیم'</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>نظارت مستمر بر شیت ۱ و داشبورد وب War Room
-خروجی: چراغ سبز ارسال رسمی و تسهیل دسترسی‌های کلان</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>بررسی روزانه ساعت ۱۶:۰۰ و تعیین تکلیف پیش‌نویس‌های آماده‌شده</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>سرکار خانم خرسنددل (سرپرست عملیات / Operation Lead)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>• هدایت فرآیند ممیزی حساب‌ها و استخراج دقیق پروفایل‌های مدیران در لینکدین
+• اعتبارسنجی پاشنه آشیل پیامکی شرکت‌ها و تحلیل ترافیک تراکنشی رقبا
+• هدایت ادمین عملیات در تدوین محتوا و مستندات فنی متناسب با هر لید
+• انتقال کارت‌های ارزیابی‌شده به مرحله تدوین نامه</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LinkedIn Sales Navigator، بورد کانبان، شیت ۲ (درخت تصمیم‌گیران)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ممیزی روزانه ۲ حساب هدف و تکمیل اطلاعات لینکدین</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>سرکار خانم فائزه (ادمین عملیات / Operation Admin)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>• تنظیم پیش‌نویس نامه‌های رسمی، پروپوزال‌های تجاری و پیام‌های InMail
+• شخصی‌سازی قلاب‌های متنی بر اساس راهکارهای فنی درگاه فِرِستا
+• ثبت و پیوست اسناد در بورد آنلاین و به‌روزرسانی لحظه‌ای وضعیت‌ها در اکسل
+• آماده‌سازی بسته‌های تستی ۵۰ هزارتایی جهت تحویل به مشتری</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Microsoft Word، ماژول اسناد بورد War Room، قالب‌های مکاتبات اداری</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>نگارش روزانه ۲ نامه رسمی و ثبت کامل پیوست‌ها در سیستم</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: unassign accounts for dynamic role taking, correct name to Khorramdel, remove purple/indigo
</commit_message>
<xml_diff>
--- a/public/pfg_b2b_tracker.xlsx
+++ b/public/pfg_b2b_tracker.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>سرپرست عملیات (خانم خرسنددل)</t>
+          <t>سرپرست عملیات (خانم خرم‌دل)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>خانم خرسنددل (Operation Lead)</t>
+          <t>خانم خرم‌دل (Operation Lead)</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -2488,7 +2488,7 @@
     <row r="5" ht="55" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
-          <t>سرکار خانم خرسنددل (سرپرست عملیات / Operation Lead)</t>
+          <t>سرکار خانم خرم‌دل (سرپرست عملیات / Operation Lead)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>